<commit_message>
data: 옵션 C — difficulty='irrelevance' 10건을 'easy'에 통합 + 본문 수치 정합화
벤치마크 데이터 (10건 라벨 통일):
- cases_analyze_network.json: 3건 (an_irr_005~007)
- cases_get_statistics.json: 3건 (gs_irr_003~005)
- cases_query_transactions.json: 4건 (qt_irr_005~008)
- benchmark_dataset.xlsx: '벤치마크 케이스' sheet difficulty 컬럼 10건

→ 4 difficulty (easy/medium/hard/irrelevance) → 3 difficulty 통일
→ Total 1258 cases 그대로 (easy 663+10=673)

Figure:
- generate_new_figures.py: difficulty list에서 'irrelevance' 제거
- fig_difficulty_distribution.png 재생성
- fig_difficulty_distribution_summary.png 재생성

본문 수치 검증 + 정합화:
- §4.5 RQ4: easy 0.799 → 0.793 (10건 흡수로 case-level 평균 미세 변동)
- 다른 difficulty 수치(medium 0.756 / hard 0.804) 변동 없음
- 카테고리별 수치 (val_str 0.289, glossary 0.525, det_aml 0.665, rank 0.888 등) 모두 정합 ✓
- 모델별 수치 영향 없음 ✓
- 'hard>medium 역전' finding 그대로 유효 ✓

근거: 'irrelevance' 10건이 categorical 분류 체계 복잡도를 증가시키는 요소
(absolute irrelevance vs domain distractor 두 abstain 난이도 분리는 paper narrative에서 활용 안 됨)
</commit_message>
<xml_diff>
--- a/benchmarks/benchmark_dataset.xlsx
+++ b/benchmarks/benchmark_dataset.xlsx
@@ -7263,7 +7263,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -21523,7 +21523,7 @@
       </c>
       <c r="C341" s="28" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D341" s="28" t="inlineStr">
@@ -21575,7 +21575,7 @@
       </c>
       <c r="C342" s="28" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D342" s="28" t="inlineStr">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="C343" s="28" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D343" s="28" t="inlineStr">
@@ -22187,7 +22187,7 @@
       </c>
       <c r="C354" s="28" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D354" s="28" t="inlineStr">
@@ -24771,7 +24771,7 @@
       </c>
       <c r="C407" s="32" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D407" s="32" t="inlineStr">
@@ -24823,7 +24823,7 @@
       </c>
       <c r="C408" s="32" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D408" s="32" t="inlineStr">
@@ -24875,7 +24875,7 @@
       </c>
       <c r="C409" s="32" t="inlineStr">
         <is>
-          <t>irrelevance</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D409" s="32" t="inlineStr">

</xml_diff>

<commit_message>
data(xlsx): rebuild 도구 정의 + 평가 시나리오 to 4-subdomain taxonomy
- 도구 정의: relabel sub domain per tool to new 4 subdomains (English,
  matching paper/README); append 3 missing Regulatory Reporting tools
  (lookup_fiu_reference_types, validate_str_fields, get_aml_glossary) ->
  23 tools, 7/4/7/5
- 평가 시나리오: relabel sub domain per row by its ground-truth function
</commit_message>
<xml_diff>
--- a/benchmarks/benchmark_dataset.xlsx
+++ b/benchmarks/benchmark_dataset.xlsx
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Regulatory Reporting</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>CTR·위험평가·모니터링</t>
+          <t>Regulatory Reporting</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>CTR·위험평가·모니터링</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>CTR·위험평가·모니터링</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>자금 흐름·추세·채널 분석</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -3474,6 +3474,57 @@
         </is>
       </c>
       <c r="I82" s="3" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Regulatory Reporting</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>FIU 의심거래 참고유형 조회 (① 정답 도구)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>lookup_fiu_reference_types</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Regulatory Reporting</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>STR 초안 필드 공식 양식 검증 (① 정답 도구)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>validate_str_fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Regulatory Reporting</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>AML 용어집 조회: CDD, STR, CTR, PEP 등 (① 정답 도구)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>get_aml_glossary</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3571,7 +3622,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -3628,7 +3679,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -3685,7 +3736,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -3742,7 +3793,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -3802,7 +3853,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -3859,7 +3910,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -3916,7 +3967,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -3973,7 +4024,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -4030,7 +4081,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -4087,7 +4138,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -4147,7 +4198,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -4204,7 +4255,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Money Flow &amp; Network Analysis</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -4264,7 +4315,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -4332,7 +4383,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -4401,7 +4452,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Regulatory Reporting</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -4461,7 +4512,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -4525,7 +4576,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -4589,7 +4640,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -4646,7 +4697,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>이상거래 통계 및 현황 조회</t>
+          <t>Transaction Inquiry &amp; Statistics</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -4703,7 +4754,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -4760,7 +4811,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Suspicious Activity Detection</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -4820,7 +4871,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>AML 탐지·분석 및 보고서 작성</t>
+          <t>Regulatory Reporting</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">

</xml_diff>